<commit_message>
iOS/Blackjack polish and Honeycomb deal-flip fixes; doc + tooling updates
Localizes remaining iOS touch-view strings (game banners, bet/dealer
labels) via tools/append_localization.py. Reworks the Blackjack result
banner to store a language-agnostic outcome instead of pre-baked text,
fixing a stale-banner-on-language-switch bug and restoring per-hand
detail for split rounds. Fixes the Honeycomb deal-flip animation, which
only ever played on the very first match of a session and skipped the
opponent's hand even then; extracts the flip/lift animation structs
(previously duplicated per-platform) into shared/Honeycomb/Views.
Restores a Windows-only localization key that had been dropped,
re-added through the xlsx pipeline instead of by hand. Documents the
banner-content workflow in mac/CLAUDE.md and adds a dev script for
launching the iOS Simulator build.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F664"/>
+  <dimension ref="A1:F672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20469,6 +20469,246 @@
         </is>
       </c>
       <c r="F664" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>touch_layout_coming_soon</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Placeholder/fallback text</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Touch layout coming soon</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Diseño táctil próximamente</t>
+        </is>
+      </c>
+      <c r="F665" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>touch_blackjack_title</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Title-case game label</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Blackjack</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Blackjack</t>
+        </is>
+      </c>
+      <c r="F666" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>touch_blackjack_banner</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>All-caps banner/header label</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>BLACKJACK</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>BLACKJACK</t>
+        </is>
+      </c>
+      <c r="F667" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>touch_spider_banner</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>All-caps banner/header label</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>SPIDER</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>SPIDER</t>
+        </is>
+      </c>
+      <c r="F668" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>touch_klondike_banner</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>All-caps banner/header label</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>KLONDIKE</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>KLONDIKE</t>
+        </is>
+      </c>
+      <c r="F669" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>touch_beecell_banner</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>All-caps banner/header label</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>BEECELL</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>BEECELL</t>
+        </is>
+      </c>
+      <c r="F670" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Chrome</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>debug_banners_menu</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Mac-only dev menu title</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Banners</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Anuncios</t>
+        </is>
+      </c>
+      <c r="F671" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>ManageDecksWin</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>deck_default_name</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Windows Manage Decks: display name for the slot-0 (default) deck</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Predeterminado</t>
+        </is>
+      </c>
+      <c r="F672" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
iOS: remove search bar from Themes sheet
The magnifying-glass toolbar button and .searchable Card Back filter
were unrequested UI weight on the Themes sheet. Drop both, and the
now-unused search_a11y localization key with them.
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F681"/>
+  <dimension ref="A1:F680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19303,27 +19303,27 @@
     <row r="626">
       <c r="A626" t="inlineStr">
         <is>
-          <t>TouchViewsIOS</t>
+          <t>SlideDownMenuIOS</t>
         </is>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>search_a11y</t>
+          <t>close_menu_a11y</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>Accessibility label for the search icon in the iOS Themes full-screen sheet toolbar</t>
+          <t>iOS slide-down menu close-button accessibility label</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Close menu</t>
         </is>
       </c>
       <c r="E626" t="inlineStr">
         <is>
-          <t>Buscar</t>
+          <t>Cerrar menú</t>
         </is>
       </c>
       <c r="F626" t="b">
@@ -19338,22 +19338,22 @@
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>close_menu_a11y</t>
+          <t>menu_section_game</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>iOS slide-down menu close-button accessibility label</t>
+          <t>iOS slide-down menu Game Selection tab section header</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>Close menu</t>
+          <t>Game</t>
         </is>
       </c>
       <c r="E627" t="inlineStr">
         <is>
-          <t>Cerrar menú</t>
+          <t>Juego</t>
         </is>
       </c>
       <c r="F627" t="b">
@@ -19368,22 +19368,22 @@
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>menu_section_game</t>
+          <t>menu_section_theme</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>iOS slide-down menu Game Selection tab section header</t>
+          <t>iOS slide-down menu Themes tab felt-color section header</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>Game</t>
+          <t>Theme</t>
         </is>
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>Juego</t>
+          <t>Tema</t>
         </is>
       </c>
       <c r="F628" t="b">
@@ -19398,22 +19398,22 @@
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>menu_section_theme</t>
+          <t>menu_section_card_back</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>iOS slide-down menu Themes tab felt-color section header</t>
+          <t>iOS slide-down menu Themes tab card-back section header</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Card Back</t>
         </is>
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>Tema</t>
+          <t>Reverso de Carta</t>
         </is>
       </c>
       <c r="F629" t="b">
@@ -19428,22 +19428,22 @@
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>menu_section_card_back</t>
+          <t>menu_section_background</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>iOS slide-down menu Themes tab card-back section header</t>
+          <t>iOS slide-down menu Themes tab background section header</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Card Back</t>
+          <t>Background</t>
         </is>
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>Reverso de Carta</t>
+          <t>Fondo</t>
         </is>
       </c>
       <c r="F630" t="b">
@@ -19458,22 +19458,22 @@
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>menu_section_background</t>
+          <t>background_none_option</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>iOS slide-down menu Themes tab background section header</t>
+          <t>iOS slide-down menu: clears the custom background back to felt color</t>
         </is>
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>Background</t>
+          <t>None</t>
         </is>
       </c>
       <c r="E631" t="inlineStr">
         <is>
-          <t>Fondo</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="F631" t="b">
@@ -19488,22 +19488,22 @@
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>background_none_option</t>
+          <t>remove_card_back_alert_title</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>iOS slide-down menu: clears the custom background back to felt color</t>
+          <t>iOS slide-down menu: confirm removing a custom card back</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Remove Card Back?</t>
         </is>
       </c>
       <c r="E632" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>¿Quitar Reverso de Carta?</t>
         </is>
       </c>
       <c r="F632" t="b">
@@ -19518,22 +19518,22 @@
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>remove_card_back_alert_title</t>
+          <t>remove_background_alert_title</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>iOS slide-down menu: confirm removing a custom card back</t>
+          <t>iOS slide-down menu: confirm removing a custom background</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>Remove Card Back?</t>
+          <t>Remove Background?</t>
         </is>
       </c>
       <c r="E633" t="inlineStr">
         <is>
-          <t>¿Quitar Reverso de Carta?</t>
+          <t>¿Quitar Fondo?</t>
         </is>
       </c>
       <c r="F633" t="b">
@@ -19548,22 +19548,22 @@
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>remove_background_alert_title</t>
+          <t>remove_imported_image_body</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>iOS slide-down menu: confirm removing a custom background</t>
+          <t>iOS slide-down menu: alert body, reused for both card-back and background removal</t>
         </is>
       </c>
       <c r="D634" t="inlineStr">
         <is>
-          <t>Remove Background?</t>
+          <t>This removes the imported image. It can't be undone.</t>
         </is>
       </c>
       <c r="E634" t="inlineStr">
         <is>
-          <t>¿Quitar Fondo?</t>
+          <t>Esto elimina la imagen importada. No se puede deshacer.</t>
         </is>
       </c>
       <c r="F634" t="b">
@@ -19578,22 +19578,22 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>remove_imported_image_body</t>
+          <t>statistics_nav_row</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>iOS slide-down menu: alert body, reused for both card-back and background removal</t>
+          <t>iOS slide-down menu: Statistics destination row</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
         <is>
-          <t>This removes the imported image. It can't be undone.</t>
+          <t>Statistics</t>
         </is>
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>Esto elimina la imagen importada. No se puede deshacer.</t>
+          <t>Estadísticas</t>
         </is>
       </c>
       <c r="F635" t="b">
@@ -19608,22 +19608,22 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>statistics_nav_row</t>
+          <t>how_to_play_nav_row</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>iOS slide-down menu: Statistics destination row</t>
+          <t>iOS slide-down menu: Help destination row</t>
         </is>
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Statistics</t>
+          <t>How to Play</t>
         </is>
       </c>
       <c r="E636" t="inlineStr">
         <is>
-          <t>Estadísticas</t>
+          <t>Cómo Jugar</t>
         </is>
       </c>
       <c r="F636" t="b">
@@ -19638,22 +19638,22 @@
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>how_to_play_nav_row</t>
+          <t>face_card_art_nav_row</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>iOS slide-down menu: Help destination row</t>
+          <t>iOS slide-down menu: Face Card Art destination row</t>
         </is>
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>How to Play</t>
+          <t>Face Card Art</t>
         </is>
       </c>
       <c r="E637" t="inlineStr">
         <is>
-          <t>Cómo Jugar</t>
+          <t>Arte de Carta</t>
         </is>
       </c>
       <c r="F637" t="b">
@@ -19663,27 +19663,27 @@
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
-          <t>SlideDownMenuIOS</t>
+          <t>TouchViewsIOS</t>
         </is>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>face_card_art_nav_row</t>
+          <t>touch_new_deal_label</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>iOS slide-down menu: Face Card Art destination row</t>
+          <t>iOS touch game views: New (deal) toolbar Label, Klondike/Spider/Beecell</t>
         </is>
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>Face Card Art</t>
+          <t>New</t>
         </is>
       </c>
       <c r="E638" t="inlineStr">
         <is>
-          <t>Arte de Carta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="F638" t="b">
@@ -19698,22 +19698,22 @@
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>touch_new_deal_label</t>
+          <t>touch_undo_last_move_label</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>iOS touch game views: New (deal) toolbar Label, Klondike/Spider/Beecell</t>
+          <t>iOS touch game views: Undo Last Move toolbar Label, Klondike/Spider/Beecell</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Undo Last Move</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Deshacer Última Jugada</t>
         </is>
       </c>
       <c r="F639" t="b">
@@ -19728,22 +19728,22 @@
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>touch_undo_last_move_label</t>
+          <t>touch_deal_a11y</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
         <is>
-          <t>iOS touch game views: Undo Last Move toolbar Label, Klondike/Spider/Beecell</t>
+          <t>iOS Spider touch view: stock pile accessibility label</t>
         </is>
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>Undo Last Move</t>
+          <t>Deal</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>Deshacer Última Jugada</t>
+          <t>Repartir</t>
         </is>
       </c>
       <c r="F640" t="b">
@@ -19758,22 +19758,22 @@
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>touch_deal_a11y</t>
+          <t>touch_completed_runs_a11y</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>iOS Spider touch view: stock pile accessibility label</t>
+          <t>iOS Spider touch view: completed-runs tray accessibility label</t>
         </is>
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>Deal</t>
+          <t>Completed runs</t>
         </is>
       </c>
       <c r="E641" t="inlineStr">
         <is>
-          <t>Repartir</t>
+          <t>Series completadas</t>
         </is>
       </c>
       <c r="F641" t="b">
@@ -19788,22 +19788,22 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>touch_completed_runs_a11y</t>
+          <t>touch_decks_picker_label</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>iOS Spider touch view: completed-runs tray accessibility label</t>
+          <t>iOS Beecell touch view: deck-count Picker label</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>Completed runs</t>
+          <t>Decks</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>Series completadas</t>
+          <t>Mazos</t>
         </is>
       </c>
       <c r="F642" t="b">
@@ -19818,22 +19818,22 @@
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>touch_decks_picker_label</t>
+          <t>touch_single_deck_option</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>iOS Beecell touch view: deck-count Picker label</t>
+          <t>iOS Beecell touch view: deck-count Picker option</t>
         </is>
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>Decks</t>
+          <t>Single Deck</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>Mazos</t>
+          <t>Mazo Sencillo</t>
         </is>
       </c>
       <c r="F643" t="b">
@@ -19848,7 +19848,7 @@
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>touch_single_deck_option</t>
+          <t>touch_double_deck_option</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
@@ -19858,12 +19858,12 @@
       </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>Single Deck</t>
+          <t>Double Deck</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>Mazo Sencillo</t>
+          <t>Doble Mazo</t>
         </is>
       </c>
       <c r="F644" t="b">
@@ -19878,22 +19878,22 @@
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>touch_double_deck_option</t>
+          <t>touch_suits_picker_label</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>iOS Beecell touch view: deck-count Picker option</t>
+          <t>iOS Spider touch view: suit-count Picker label (mislabeled "Difficulty" in source, corrected to match Mac's "Suits:")</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>Double Deck</t>
+          <t>Suits</t>
         </is>
       </c>
       <c r="E645" t="inlineStr">
         <is>
-          <t>Doble Mazo</t>
+          <t>Palos</t>
         </is>
       </c>
       <c r="F645" t="b">
@@ -19908,22 +19908,22 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>touch_suits_picker_label</t>
+          <t>touch_bet_max_button</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>iOS Spider touch view: suit-count Picker label (mislabeled "Difficulty" in source, corrected to match Mac's "Suits:")</t>
+          <t>iOS Video Poker touch view: Max bet button</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>Suits</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>Palos</t>
+          <t>Máx</t>
         </is>
       </c>
       <c r="F646" t="b">
@@ -19938,22 +19938,22 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>touch_bet_max_button</t>
+          <t>touch_settings_unlock_between_hands</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>iOS Video Poker touch view: Max bet button</t>
+          <t>iOS Blackjack touch view: settings-locked notice during a round</t>
         </is>
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>Max</t>
+          <t>Settings unlock between hands.</t>
         </is>
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>Máx</t>
+          <t>La configuración se desbloquea entre manos.</t>
         </is>
       </c>
       <c r="F647" t="b">
@@ -19968,22 +19968,22 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>touch_settings_unlock_between_hands</t>
+          <t>touch_settings_unlock_hand_ends</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
         <is>
-          <t>iOS Blackjack touch view: settings-locked notice during a round</t>
+          <t>iOS Video Poker touch view: settings-locked notice during a hand</t>
         </is>
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>Settings unlock between hands.</t>
+          <t>Settings unlock when the hand ends.</t>
         </is>
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>La configuración se desbloquea entre manos.</t>
+          <t>La configuración se desbloquea cuando termina la mano.</t>
         </is>
       </c>
       <c r="F648" t="b">
@@ -19998,22 +19998,22 @@
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>touch_settings_unlock_hand_ends</t>
+          <t>touch_hands_dealt_stat</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>iOS Video Poker touch view: settings-locked notice during a hand</t>
+          <t>iOS Blackjack/Video Poker touch stats: hands-dealt row label</t>
         </is>
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>Settings unlock when the hand ends.</t>
+          <t>Hands Dealt</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>La configuración se desbloquea cuando termina la mano.</t>
+          <t>Manos Repartidas</t>
         </is>
       </c>
       <c r="F649" t="b">
@@ -20028,22 +20028,22 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>touch_hands_dealt_stat</t>
+          <t>touch_session_credits_stat</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>iOS Blackjack/Video Poker touch stats: hands-dealt row label</t>
+          <t>iOS Blackjack/Video Poker touch stats: session-credits row label</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>Hands Dealt</t>
+          <t>Session Credits</t>
         </is>
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>Manos Repartidas</t>
+          <t>Créditos de Sesión</t>
         </is>
       </c>
       <c r="F650" t="b">
@@ -20058,22 +20058,22 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>touch_session_credits_stat</t>
+          <t>touch_hand_label_fmt</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>iOS Blackjack/Video Poker touch stats: session-credits row label</t>
+          <t>iOS Blackjack touch view: per-hand label when split (multiple hands), %d is the hand number</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>Session Credits</t>
+          <t>HAND %d</t>
         </is>
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>Créditos de Sesión</t>
+          <t>MANO %d</t>
         </is>
       </c>
       <c r="F651" t="b">
@@ -20088,22 +20088,22 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>touch_hand_label_fmt</t>
+          <t>touch_you_label</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>iOS Blackjack touch view: per-hand label when split (multiple hands), %d is the hand number</t>
+          <t>iOS Blackjack touch view: player hand label when not split (single hand)</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>HAND %d</t>
+          <t>YOU</t>
         </is>
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>MANO %d</t>
+          <t>TÚ</t>
         </is>
       </c>
       <c r="F652" t="b">
@@ -20118,22 +20118,22 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>touch_you_label</t>
+          <t>touch_bust_suffix</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>iOS Blackjack touch view: player hand label when not split (single hand)</t>
+          <t>iOS Blackjack touch view: appended to a hand value when busted (leading space intentional)</t>
         </is>
       </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>YOU</t>
+          <t xml:space="preserve"> BUST</t>
         </is>
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>TÚ</t>
+          <t xml:space="preserve"> SE PASÓ</t>
         </is>
       </c>
       <c r="F653" t="b">
@@ -20148,22 +20148,22 @@
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>touch_bust_suffix</t>
+          <t>touch_result_win</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>iOS Blackjack touch view: appended to a hand value when busted (leading space intentional)</t>
+          <t>iOS Blackjack touch view: per-hand result badge</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BUST</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SE PASÓ</t>
+          <t>GANA</t>
         </is>
       </c>
       <c r="F654" t="b">
@@ -20178,7 +20178,7 @@
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>touch_result_win</t>
+          <t>touch_result_loss</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
@@ -20188,12 +20188,12 @@
       </c>
       <c r="D655" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>GANA</t>
+          <t>PIERDE</t>
         </is>
       </c>
       <c r="F655" t="b">
@@ -20208,7 +20208,7 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>touch_result_loss</t>
+          <t>touch_result_push</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
@@ -20218,12 +20218,12 @@
       </c>
       <c r="D656" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>PUSH</t>
         </is>
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>PIERDE</t>
+          <t>EMPATE</t>
         </is>
       </c>
       <c r="F656" t="b">
@@ -20238,7 +20238,7 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>touch_result_push</t>
+          <t>touch_result_blackjack</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -20248,12 +20248,12 @@
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>PUSH</t>
+          <t>BLACKJACK!</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>EMPATE</t>
+          <t>¡BLACKJACK!</t>
         </is>
       </c>
       <c r="F657" t="b">
@@ -20268,7 +20268,7 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>touch_result_blackjack</t>
+          <t>touch_result_bust</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -20278,12 +20278,12 @@
       </c>
       <c r="D658" t="inlineStr">
         <is>
-          <t>BLACKJACK!</t>
+          <t>BUST</t>
         </is>
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>¡BLACKJACK!</t>
+          <t>SE PASÓ</t>
         </is>
       </c>
       <c r="F658" t="b">
@@ -20298,22 +20298,22 @@
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>touch_result_bust</t>
+          <t>touch_action_hit</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>iOS Blackjack touch view: per-hand result badge</t>
+          <t>iOS Blackjack touch view: action button</t>
         </is>
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>BUST</t>
+          <t>Hit</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>SE PASÓ</t>
+          <t>Pedir</t>
         </is>
       </c>
       <c r="F659" t="b">
@@ -20328,7 +20328,7 @@
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>touch_action_hit</t>
+          <t>touch_action_stand</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
@@ -20338,12 +20338,12 @@
       </c>
       <c r="D660" t="inlineStr">
         <is>
-          <t>Hit</t>
+          <t>Stand</t>
         </is>
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>Pedir</t>
+          <t>Plantarse</t>
         </is>
       </c>
       <c r="F660" t="b">
@@ -20358,7 +20358,7 @@
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>touch_action_stand</t>
+          <t>touch_action_double</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
@@ -20368,12 +20368,12 @@
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>Stand</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>Plantarse</t>
+          <t>Doblar</t>
         </is>
       </c>
       <c r="F661" t="b">
@@ -20388,7 +20388,7 @@
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>touch_action_double</t>
+          <t>touch_action_split</t>
         </is>
       </c>
       <c r="C662" t="inlineStr">
@@ -20398,12 +20398,12 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>Split</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>Doblar</t>
+          <t>Dividir</t>
         </is>
       </c>
       <c r="F662" t="b">
@@ -20418,22 +20418,22 @@
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>touch_action_split</t>
+          <t>touch_reset_position_button</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>iOS Blackjack touch view: action button</t>
+          <t>iOS custom-art import sheets: Reset Position button</t>
         </is>
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Reset Position</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>Dividir</t>
+          <t>Restablecer Posición</t>
         </is>
       </c>
       <c r="F663" t="b">
@@ -20448,22 +20448,22 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>touch_reset_position_button</t>
+          <t>touch_add_card_back_title</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: Reset Position button</t>
+          <t>iOS custom card-back import sheet nav title</t>
         </is>
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>Reset Position</t>
+          <t>Add Card Back</t>
         </is>
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>Restablecer Posición</t>
+          <t>Añadir Reverso de Carta</t>
         </is>
       </c>
       <c r="F664" t="b">
@@ -20473,27 +20473,29 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>TouchViewsIOS</t>
+          <t>Honeycomb</t>
         </is>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>touch_add_card_back_title</t>
+          <t>steal_instruction_tap</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>iOS custom card-back import sheet nav title</t>
+          <t>Steal-mode instructional hint, iOS (touch wording — Mac/Windows use the click-based steal_instruction key)</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>Add Card Back</t>
+          <t>Double-tap a captured opponent's card
+on the board to steal it.</t>
         </is>
       </c>
       <c r="E665" t="inlineStr">
         <is>
-          <t>Añadir Reverso de Carta</t>
+          <t>Toca dos veces la carta capturada de un oponente
+en el tablero para robarla.</t>
         </is>
       </c>
       <c r="F665" t="b">
@@ -20503,29 +20505,27 @@
     <row r="666">
       <c r="A666" t="inlineStr">
         <is>
-          <t>Honeycomb</t>
+          <t>TouchViewsIOS</t>
         </is>
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>steal_instruction_tap</t>
+          <t>touch_layout_coming_soon</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>Steal-mode instructional hint, iOS (touch wording — Mac/Windows use the click-based steal_instruction key)</t>
+          <t>Placeholder/fallback text</t>
         </is>
       </c>
       <c r="D666" t="inlineStr">
         <is>
-          <t>Double-tap a captured opponent's card
-on the board to steal it.</t>
+          <t>Touch layout coming soon</t>
         </is>
       </c>
       <c r="E666" t="inlineStr">
         <is>
-          <t>Toca dos veces la carta capturada de un oponente
-en el tablero para robarla.</t>
+          <t>Diseño táctil próximamente</t>
         </is>
       </c>
       <c r="F666" t="b">
@@ -20540,26 +20540,26 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>touch_layout_coming_soon</t>
+          <t>touch_blackjack_title</t>
         </is>
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>Placeholder/fallback text</t>
+          <t>Title-case game label</t>
         </is>
       </c>
       <c r="D667" t="inlineStr">
         <is>
-          <t>Touch layout coming soon</t>
+          <t>Blackjack</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>Diseño táctil próximamente</t>
+          <t>Blackjack</t>
         </is>
       </c>
       <c r="F667" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="668">
@@ -20570,22 +20570,22 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>touch_blackjack_title</t>
+          <t>touch_blackjack_banner</t>
         </is>
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>Title-case game label</t>
+          <t>All-caps banner/header label</t>
         </is>
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>Blackjack</t>
+          <t>BLACKJACK</t>
         </is>
       </c>
       <c r="E668" t="inlineStr">
         <is>
-          <t>Blackjack</t>
+          <t>BLACKJACK</t>
         </is>
       </c>
       <c r="F668" t="b">
@@ -20600,7 +20600,7 @@
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>touch_blackjack_banner</t>
+          <t>touch_spider_banner</t>
         </is>
       </c>
       <c r="C669" t="inlineStr">
@@ -20610,12 +20610,12 @@
       </c>
       <c r="D669" t="inlineStr">
         <is>
-          <t>BLACKJACK</t>
+          <t>SPIDER</t>
         </is>
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>BLACKJACK</t>
+          <t>SPIDER</t>
         </is>
       </c>
       <c r="F669" t="b">
@@ -20630,7 +20630,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>touch_spider_banner</t>
+          <t>touch_klondike_banner</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
@@ -20640,12 +20640,12 @@
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>SPIDER</t>
+          <t>KLONDIKE</t>
         </is>
       </c>
       <c r="E670" t="inlineStr">
         <is>
-          <t>SPIDER</t>
+          <t>KLONDIKE</t>
         </is>
       </c>
       <c r="F670" t="b">
@@ -20660,7 +20660,7 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>touch_klondike_banner</t>
+          <t>touch_beecell_banner</t>
         </is>
       </c>
       <c r="C671" t="inlineStr">
@@ -20670,12 +20670,12 @@
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>KLONDIKE</t>
+          <t>BEECELL</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>KLONDIKE</t>
+          <t>BEECELL</t>
         </is>
       </c>
       <c r="F671" t="b">
@@ -20685,57 +20685,57 @@
     <row r="672">
       <c r="A672" t="inlineStr">
         <is>
-          <t>TouchViewsIOS</t>
+          <t>Chrome</t>
         </is>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>touch_beecell_banner</t>
+          <t>debug_banners_menu</t>
         </is>
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>All-caps banner/header label</t>
+          <t>Mac-only dev menu title</t>
         </is>
       </c>
       <c r="D672" t="inlineStr">
         <is>
-          <t>BEECELL</t>
+          <t>Banners</t>
         </is>
       </c>
       <c r="E672" t="inlineStr">
         <is>
-          <t>BEECELL</t>
+          <t>Anuncios</t>
         </is>
       </c>
       <c r="F672" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr">
         <is>
-          <t>Chrome</t>
+          <t>ManageDecksWin</t>
         </is>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>debug_banners_menu</t>
+          <t>deck_default_name</t>
         </is>
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>Mac-only dev menu title</t>
+          <t>Windows Manage Decks: display name for the slot-0 (default) deck</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>Banners</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="E673" t="inlineStr">
         <is>
-          <t>Anuncios</t>
+          <t>Predeterminado</t>
         </is>
       </c>
       <c r="F673" t="b">
@@ -20745,27 +20745,27 @@
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>ManageDecksWin</t>
+          <t>TouchViewsIOS</t>
         </is>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>deck_default_name</t>
+          <t>free_play_label</t>
         </is>
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>Windows Manage Decks: display name for the slot-0 (default) deck</t>
+          <t>iOS Blackjack/Video Poker touch view: credits capsule label in free-play mode</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Free Play</t>
         </is>
       </c>
       <c r="E674" t="inlineStr">
         <is>
-          <t>Predeterminado</t>
+          <t>Juego Libre</t>
         </is>
       </c>
       <c r="F674" t="b">
@@ -20780,22 +20780,22 @@
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>free_play_label</t>
+          <t>touch_choose_photo</t>
         </is>
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>iOS Blackjack/Video Poker touch view: credits capsule label in free-play mode</t>
+          <t>iOS custom-art import sheets: photo picker button, no image chosen yet</t>
         </is>
       </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>Free Play</t>
+          <t>Choose Photo</t>
         </is>
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>Juego Libre</t>
+          <t>Elegir Foto</t>
         </is>
       </c>
       <c r="F675" t="b">
@@ -20810,22 +20810,22 @@
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>touch_choose_photo</t>
+          <t>touch_choose_different_photo</t>
         </is>
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: photo picker button, no image chosen yet</t>
+          <t>iOS custom-art import sheets: photo picker button, image already chosen</t>
         </is>
       </c>
       <c r="D676" t="inlineStr">
         <is>
-          <t>Choose Photo</t>
+          <t>Choose a Different Photo</t>
         </is>
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>Elegir Foto</t>
+          <t>Elegir Otra Foto</t>
         </is>
       </c>
       <c r="F676" t="b">
@@ -20840,22 +20840,22 @@
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>touch_choose_different_photo</t>
+          <t>touch_pinch_zoom_reposition</t>
         </is>
       </c>
       <c r="C677" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: photo picker button, image already chosen</t>
+          <t>iOS custom-art import sheets: crop editor section header</t>
         </is>
       </c>
       <c r="D677" t="inlineStr">
         <is>
-          <t>Choose a Different Photo</t>
+          <t>Pinch to zoom, drag to reposition</t>
         </is>
       </c>
       <c r="E677" t="inlineStr">
         <is>
-          <t>Elegir Otra Foto</t>
+          <t>Pellizca para hacer zoom, arrastra para reposicionar</t>
         </is>
       </c>
       <c r="F677" t="b">
@@ -20870,22 +20870,22 @@
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>touch_pinch_zoom_reposition</t>
+          <t>touch_name_field_placeholder</t>
         </is>
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: crop editor section header</t>
+          <t>iOS custom-art import sheets: name TextField placeholder</t>
         </is>
       </c>
       <c r="D678" t="inlineStr">
         <is>
-          <t>Pinch to zoom, drag to reposition</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>Pellizca para hacer zoom, arrastra para reposicionar</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="F678" t="b">
@@ -20900,22 +20900,22 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>touch_name_field_placeholder</t>
+          <t>touch_name_already_taken_error</t>
         </is>
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: name TextField placeholder</t>
+          <t>iOS custom-art import sheets: duplicate-name validation error</t>
         </is>
       </c>
       <c r="D679" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>That name is already taken — pick another.</t>
         </is>
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>Nombre</t>
+          <t>Ese nombre ya está en uso — elige otro.</t>
         </is>
       </c>
       <c r="F679" t="b">
@@ -20930,55 +20930,25 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>touch_name_already_taken_error</t>
+          <t>touch_enabled_toggle</t>
         </is>
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>iOS custom-art import sheets: duplicate-name validation error</t>
+          <t>iOS custom face-card-art import sheet: Enabled toggle label</t>
         </is>
       </c>
       <c r="D680" t="inlineStr">
         <is>
-          <t>That name is already taken — pick another.</t>
+          <t>Enabled</t>
         </is>
       </c>
       <c r="E680" t="inlineStr">
         <is>
-          <t>Ese nombre ya está en uso — elige otro.</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="F680" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="681">
-      <c r="A681" t="inlineStr">
-        <is>
-          <t>TouchViewsIOS</t>
-        </is>
-      </c>
-      <c r="B681" t="inlineStr">
-        <is>
-          <t>touch_enabled_toggle</t>
-        </is>
-      </c>
-      <c r="C681" t="inlineStr">
-        <is>
-          <t>iOS custom face-card-art import sheet: Enabled toggle label</t>
-        </is>
-      </c>
-      <c r="D681" t="inlineStr">
-        <is>
-          <t>Enabled</t>
-        </is>
-      </c>
-      <c r="E681" t="inlineStr">
-        <is>
-          <t>Activado</t>
-        </is>
-      </c>
-      <c r="F681" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
iOS: auto-name new card backs "Default"/"Default N", name field to top
Add Card Back no longer requires typing a name to save — the Name
field moves above the photo picker and is pre-filled with the first
free "Default"/"Default 1"/"Default 2"... slot. Tapping into the field
clears the auto-filled value so the player gets a blank space to type
a real name, rather than having to select-all first.
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F680"/>
+  <dimension ref="A1:F681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20949,6 +20949,36 @@
         </is>
       </c>
       <c r="F680" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>card_back_default_name</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Auto-filled base name for a new custom card back before the user renames it (appended with ' N' for the 2nd, 3rd, ... duplicate)</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Predeterminado</t>
+        </is>
+      </c>
+      <c r="F681" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Spanish help strings for hotkeys and strategy title
Arrow Keys/Space now read "Flechas del Teclado" / "Barra espaciadora",
and the strategy section title drops the redundant "Pro" to just
"Estrategia y consejos".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -14139,7 +14139,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>💡 Estrategia y Consejos Pro</t>
+          <t>💡 Estrategia y consejos</t>
         </is>
       </c>
       <c r="F457" t="b">
@@ -14409,7 +14409,7 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>Teclas de Flecha</t>
+          <t>Flechas del Teclado</t>
         </is>
       </c>
       <c r="F466" t="b">
@@ -14469,7 +14469,7 @@
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>Espacio / Intro</t>
+          <t>Barra espaciadora / Intro</t>
         </is>
       </c>
       <c r="F468" t="b">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="E527" t="inlineStr">
         <is>
-          <t>Teclas de Flecha + Espacio / Intro</t>
+          <t>Flechas del Teclado + Barra espaciadora / Intro</t>
         </is>
       </c>
       <c r="F527" t="b">

</xml_diff>

<commit_message>
iOS: fix truncated/generic tile captions in Themes Background grid
"Custom Felt Color" was truncating to "Custom Felt.." at the tile's
narrow width; add a dedicated shorter string. The Add-background tile
reused the generic "Add" caption shared with Card Backs/Face Art's
plain-add tiles — give it "Add Photo" instead since this one specifically
imports a photo.
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F681"/>
+  <dimension ref="A1:F683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20979,6 +20979,66 @@
         </is>
       </c>
       <c r="F681" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>add_photo_short</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Caption on the iOS Themes sheet Background grid's Add tile (imports a photo, unlike Card Back/Face Art's plain "Add")</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Add Photo</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Añadir Foto</t>
+        </is>
+      </c>
+      <c r="F682" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>felt_custom_short</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Caption on the iOS Themes sheet Background grid's Custom Felt tile — shorter than feltCustomColor ("Custom Felt Color") so it fits the narrow tile without truncating</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Custom Felt</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Fieltro Personalizado</t>
+        </is>
+      </c>
+      <c r="F683" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
iOS Honeycomb: add stat-filter dropdowns to Card Bank, mirroring mac's freeform search
Mac lets you type a value onto a mini card graphic per corner
(Top/Right/Bottom/Left) to filter the card bank, with an exact match
at full opacity and a +/-2 tolerance match dimmed to 40%. No room for
that widget on a phone, so this adds four dropdowns (1-9, A) instead,
replicating the same AND-across-filled-fields / exact-vs-near dimming
logic. Scoped to the main Card Bank browse grid only, same as mac —
Deck Builder's embedded grid is unaffected.
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F683"/>
+  <dimension ref="A1:F688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21039,6 +21039,156 @@
         </is>
       </c>
       <c r="F683" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>stat_position_top</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's top corner value</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Arriba</t>
+        </is>
+      </c>
+      <c r="F684" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>stat_position_bottom</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's bottom corner value</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Abajo</t>
+        </is>
+      </c>
+      <c r="F685" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>stat_position_left</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's left corner value</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Izquierda</t>
+        </is>
+      </c>
+      <c r="F686" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>stat_position_right</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Label on the iOS Card Bank stat-filter dropdown for a card's right corner value</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Derecha</t>
+        </is>
+      </c>
+      <c r="F687" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>TouchViewsIOS</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>stat_filter_any</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Default/unset option in each iOS Card Bank stat-filter dropdown (matches any value)</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Cualquiera</t>
+        </is>
+      </c>
+      <c r="F688" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Honeycomb iOS: score badge shows opponent's name, rules banner gets mac's boxed styling
- score_dealer_fmt was a fixed "%d DEALER" template; changed to "%d %@"
  and pass honeycombLocalizedDifficultyName at the call site, so the
  score badge reads "5 Baby Bee" instead of "5 DEALER" (same fix as the
  hand-side label and opponent-name work earlier this session).
- The pre-game/mid-match rules line ("Roulette", "Normal", etc.) was
  bare yellow text with no background, unlike mac's dedicated "Rules:"
  title + value card on a solid black.opacity(0.75) rounded box. Now
  wrapped in the same treatment, sized down to fit alongside the
  hint/undo buttons; bannerRowHeight bumped 46->58 to fit the two lines
  (intrinsicSize(landscape:) already keys off this constant, so layout
  stays in sync automatically).
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -4317,17 +4317,17 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Score badge, %d = dealer score — Honeycomb touch view</t>
+          <t>Score badge, Honeycomb touch view — %d = opponent score, %@/{1} = opponent's difficulty name (e.g. Baby Bee)</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>%d DEALER</t>
+          <t>%d %@</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>%d REPARTIDOR</t>
+          <t>%d %@</t>
         </is>
       </c>
       <c r="F130" t="b">

</xml_diff>

<commit_message>
Solitaire: center score capsule on top bar; Honeycomb: "You" instead of "YOU"
Klondike/Beecell/Spider top bars now overlay the SCORE/TIME capsule on
the full bar width instead of centering it in the leftover space
between the (differently-sized) menu and New Deal button groups.

Also normalizes the Honeycomb score badge to sentence case ("You 5 -
5 Baby Bee") to match the rest of the UI, in English and Spanish.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -4292,12 +4292,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>YOU %d</t>
+          <t>You %d</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>TÚ %d</t>
+          <t>Tú %d</t>
         </is>
       </c>
       <c r="F129" t="b">

</xml_diff>

<commit_message>
Fix Honeycomb crash from mismatched score format string + flip-state resync
scoreDealerFmt was "%d %@" (int first, object second) in the localization
catalog, but the call site passes (name: String, score: Int) — the %@
placeholder ended up trying to message the Int as if it were an object
pointer, crashing (SIGSEGV) every time the Honeycomb score capsule
rendered. Fixed via the xlsx source and regeneration to "%@ %d",
matching the actual call order.

Also fixes cards staying stuck face-down and unplayable after switching
away from Honeycomb mid-match and back: IOSRouterView's switch on
gameMode fully unmounts HoneycombTouchView (unlike mac, which keeps
every game's view alive at once), resetting its flip-reveal @State to
all-false while the underlying view model — unreset — stays mid-match.
onAppear now resyncs the reveal state with reality when returning to an
already-.playing/.suddenDeath match.
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -4317,17 +4317,17 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Score badge, Honeycomb touch view — %d = opponent score, %@/{1} = opponent's difficulty name (e.g. Baby Bee)</t>
+          <t>Score badge, Honeycomb touch view — %@/{0} = opponent's difficulty name (e.g. Baby Bee), %d = opponent score</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>%d %@</t>
+          <t>%@ %d</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>%d %@</t>
+          <t>%@ %d</t>
         </is>
       </c>
       <c r="F130" t="b">

</xml_diff>

<commit_message>
Add bee watermark with Hide the Bee toggle across iOS, macOS, and Windows
Draws a centered bee watermark behind every game's board, with a global
"Hide the Bee" toggle and a temporary per-game calibration slider that
live-saves scale while the right values get dialed in. Also caps
Windows' board content scale at 2.0x to match mac's existing zoom cap.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F684"/>
+  <dimension ref="A1:F685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21069,6 +21069,36 @@
         </is>
       </c>
       <c r="F684" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>hide_bee</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Toggle label, reused across every game's Options on Mac/iOS/Windows</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Hide the Bee</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Ocultar la Abeja</t>
+        </is>
+      </c>
+      <c r="F685" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename Honey Mode to Enable Banners in localization
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -1500,12 +1500,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Honey Mode (Flavor)</t>
+          <t>Enable Banners</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Modo Miel (Sabor)</t>
+          <t>Activar Anuncios</t>
         </is>
       </c>
       <c r="F36" t="b">
@@ -15142,14 +15142,14 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>• Honey Mode (Flavor): Global toggle across all 6 games — controls the "+N"/"-N" score popups and whether flavor/ambiance banners appear. Turn it off for a quieter, more minimal play experience.
+          <t>• Enable Banners: Global toggle across all 6 games — controls the "+N"/"-N" score popups and whether flavor/ambiance banners appear. Turn it off for a quieter, more minimal play experience.
 • Stay on Top: Keeps the game window pinned above your other windows (View menu).
 • Sound Effects, Vegas Scoring, and Hide Hint Button are also available here per-game.</t>
         </is>
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>• Modo Miel (Sabor): Interruptor global en los 6 juegos — controla las ventanas emergentes de puntuación "+N"/"-N" y si aparecen los carteles de sabor/ambiente. Desactívalo para una experiencia de juego más silenciosa y minimalista.
+          <t>• Activar Anuncios: Interruptor global en los 6 juegos — controla las ventanas emergentes de puntuación "+N"/"-N" y si aparecen los carteles de sabor/ambiente. Desactívalo para una experiencia de juego más silenciosa y minimalista.
 • Siempre Encima: Mantiene la ventana del juego anclada sobre tus otras ventanas (Menú Vista).
 • Efectos de Sonido, Puntuación Vegas, y Ocultar Botón de Pistas también están disponibles aquí por juego.</t>
         </is>

</xml_diff>

<commit_message>
Add Honeycomb player-rank and toggle-tooltip localization keys
Restores rank_* and *_tooltip keys from the xlsx source of truth (they'd
been hand-edited directly into the generated Swift/C# files earlier and
were silently dropped by a subsequent regeneration), fixes hand_label_you
capitalization ("YOU" -> "You"), and keeps the Honey Mode toggle labeled
"Honey Mode" rather than "Enable Banners". Also updates the iOS stacked
betting-grid Clear button to reference the surviving btn_clear_short key
instead of the removed btn_clear.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F685"/>
+  <dimension ref="A1:F697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1500,12 +1500,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Enable Banners</t>
+          <t>Honey Mode</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Activar Anuncios</t>
+          <t>Modo Miel</t>
         </is>
       </c>
       <c r="F36" t="b">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>YOU</t>
+          <t>You</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -15142,14 +15142,14 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>• Enable Banners: Global toggle across all 6 games — controls the "+N"/"-N" score popups and whether flavor/ambiance banners appear. Turn it off for a quieter, more minimal play experience.
+          <t>• Honey Mode: Global toggle across all 6 games — controls the "+N"/"-N" score popups and whether flavor/ambiance banners appear. Turn it off for a quieter, more minimal play experience.
 • Stay on Top: Keeps the game window pinned above your other windows (View menu).
 • Sound Effects, Vegas Scoring, and Hide Hint Button are also available here per-game.</t>
         </is>
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>• Activar Anuncios: Interruptor global en los 6 juegos — controla las ventanas emergentes de puntuación "+N"/"-N" y si aparecen los carteles de sabor/ambiente. Desactívalo para una experiencia de juego más silenciosa y minimalista.
+          <t>• Modo Miel: Interruptor global en los 6 juegos — controla las ventanas emergentes de puntuación "+N"/"-N" y si aparecen los carteles de sabor/ambiente. Desactívalo para una experiencia de juego más silenciosa y minimalista.
 • Siempre Encima: Mantiene la ventana del juego anclada sobre tus otras ventanas (Menú Vista).
 • Efectos de Sonido, Puntuación Vegas, y Ocultar Botón de Pistas también están disponibles aquí por juego.</t>
         </is>
@@ -21099,6 +21099,366 @@
         </is>
       </c>
       <c r="F685" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>honey_mode_tooltip</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Tooltip for the Honey Mode toggle</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Enables banners and solitaire point animations.</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Habilita los anuncios y las animaciones de puntos en los solitarios.</t>
+        </is>
+      </c>
+      <c r="F686" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>no_stress_mode_tooltip</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Tooltip for the No Stress Mode toggle</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Pressure-free! No timers, no betting, and Honeycomb chooses your deck for you at random.</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>¡Sin presión! Sin temporizadores, sin apuestas, y Honeycomb elige tu mazo al azar.</t>
+        </is>
+      </c>
+      <c r="F687" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>rank_nurse_bee</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Player rank, 10-19 cards collected</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Nurse Bee</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Abeja Nodriza</t>
+        </is>
+      </c>
+      <c r="F688" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>rank_scout_bee</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Player rank, 20-49 cards collected</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Scout Bee</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Abeja Exploradora</t>
+        </is>
+      </c>
+      <c r="F689" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>rank_worker_bee</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Player rank, 50-99 cards collected</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Worker Bee</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Abeja Obrera</t>
+        </is>
+      </c>
+      <c r="F690" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>rank_guard_bee</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Player rank, 100-149 cards collected</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Guard Bee</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Abeja Guardiana</t>
+        </is>
+      </c>
+      <c r="F691" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>rank_waggle_dancer</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Player rank, 150-199 cards collected</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Waggle Dancer</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Abeja Bailarina</t>
+        </is>
+      </c>
+      <c r="F692" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>rank_comb_architect</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Player rank, 200-299 cards collected</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Comb Architect</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Arquitecta del Panal</t>
+        </is>
+      </c>
+      <c r="F693" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>rank_royal_attendant</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Player rank, 300-399 cards collected</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Royal Attendant</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Asistente Real</t>
+        </is>
+      </c>
+      <c r="F694" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>rank_swarm_leader</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Player rank, 400-499 cards collected</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Swarm Leader</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Líder del Enjambre</t>
+        </is>
+      </c>
+      <c r="F695" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>rank_hive_monarch</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Player rank, 500+ cards collected but not the full set</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Hive Monarch</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Monarca de la Colmena</t>
+        </is>
+      </c>
+      <c r="F696" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Honeycomb</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>rank_apiarist</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Player rank, every card in the collection unlocked</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Apiarist</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Apicultor</t>
+        </is>
+      </c>
+      <c r="F697" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Spider help (Spanish): "prefiere" -> "prioriza" in strategy tip #1
Also restores the global_settings_header key to the xlsx source of truth
— a prior commit had hand-added it directly to the generated Windows
Strings.cs/StringKey.cs (bypassing the xlsx), so it would have been
silently dropped by the next full regeneration.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F697"/>
+  <dimension ref="A1:F698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14671,7 +14671,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>1. Mismo Palo Antes que Palos Mixtos: Siempre prefiere construir rachas del mismo palo. Las pilas de palos mixtos bloquean tus cartas y no pueden moverse juntas.
+          <t>1. Mismo Palo Antes que Palos Mixtos: Siempre prioriza construir rachas del mismo palo. Las pilas de palos mixtos bloquean tus cartas y no pueden moverse juntas.
 2. Columnas Vacías Primero: Las columnas vacías te permiten aislar pilas de palos mixtos y reorganizarlas en limpias rachas del mismo palo.
 3. Retrasa el Reparto: Agota cada movimiento posible en el tablero antes de hacer clic en la pila.</t>
         </is>
@@ -21459,6 +21459,36 @@
         </is>
       </c>
       <c r="F697" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>global_settings_header</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Section header, Windows Preferences panel — global (cross-game) settings group</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Global Settings</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Configuración Global</t>
+        </is>
+      </c>
+      <c r="F698" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix cross-platform localization drift for stats/dialogs, drop two Windows-only confirmations
- Align "Win Rate" text on mac/Windows to match iOS across Klondike/Beecell/Spider
- Fix iOS Spider to use the shared avg-winning-time key instead of a stray one-off
- Route Windows' New Game / Restart confirmation dialogs through the shared
  localization keys instead of hardcoded English, and align the Restart button
  text with mac's "Restart Game"
- Fix Windows VideoPoker's Clear-Holds shortcut to [C], matching mac (was [Q])
- Remove the Windows-only "Change Game Mode?" and "Switch Variant?" confirmation
  popups entirely so those actions apply immediately, matching iOS's behavior

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -2250,12 +2250,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Win Percentage</t>
+          <t>Win Rate</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Porcentaje de Victorias</t>
+          <t>Tasa de Victorias</t>
         </is>
       </c>
       <c r="F61" t="b">
@@ -4172,12 +4172,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Rebuy</t>
+          <t>Buy In</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Recomprar</t>
+          <t>Comprar Fichas</t>
         </is>
       </c>
       <c r="F125" t="b">
@@ -5944,12 +5944,12 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Background, outline, text, hint highlight</t>
+          <t>Background, outline, suit text, hint highlight</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Fondo, contorno, texto, resaltado de pista</t>
+          <t>Fondo, contorno, texto de palo, resaltado de pista</t>
         </is>
       </c>
       <c r="F184" t="b">
@@ -7984,12 +7984,12 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Win Percentage:</t>
+          <t>Win Rate:</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Porcentaje de Victorias:</t>
+          <t>Tasa de Victorias:</t>
         </is>
       </c>
       <c r="F252" t="b">
@@ -8734,12 +8734,12 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>REBUY</t>
+          <t>BUY IN</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>RECOMPRAR</t>
+          <t>COMPRAR FICHAS</t>
         </is>
       </c>
       <c r="F277" t="b">
@@ -10114,12 +10114,12 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Clear  [Q]</t>
+          <t>Clear  [C]</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Borrar  [Q]</t>
+          <t>Borrar  [C]</t>
         </is>
       </c>
       <c r="F323" t="b">
@@ -11044,12 +11044,12 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>Force Normal Rules</t>
+          <t>Normal Mode (Force Zero Rules)</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Forzar Reglas Normales</t>
+          <t>Modo Normal (Forzar Cero Reglas)</t>
         </is>
       </c>
       <c r="F354" t="b">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>Honeycomb Statistics</t>
+          <t>Honeycomb Stats</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -11284,7 +11284,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>Matches Played</t>
+          <t>Games Played</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -11554,12 +11554,12 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>Flawless Victories (10-0 Sweep)</t>
+          <t>Flawless Victories</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Victorias Perfectas (Barrida 10-0)</t>
+          <t>Victorias Perfectas</t>
         </is>
       </c>
       <c r="F371" t="b">
@@ -11584,12 +11584,12 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>Same/Plus Triggers</t>
+          <t>Symmetry/Math Bee Hive Minds Triggered</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Activaciones Same/Plus</t>
+          <t>Mentes Colmena Simetría/Abeja Matemática Activadas</t>
         </is>
       </c>
       <c r="F372" t="b">
@@ -12214,12 +12214,12 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Saved Decks &amp; Card Bank</t>
+          <t>Manage Decks</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Mazos Guardados y Banco de Cartas</t>
+          <t>Administrar Mazos</t>
         </is>
       </c>
       <c r="F393" t="b">
@@ -20880,12 +20880,12 @@
       </c>
       <c r="D678" t="inlineStr">
         <is>
-          <t>Sudden Deaths</t>
+          <t>Most Swarms to the Death</t>
         </is>
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>Muertes Súbitas</t>
+          <t>Más Enjambres a Muerte</t>
         </is>
       </c>
       <c r="F678" t="b">
@@ -20910,12 +20910,12 @@
       </c>
       <c r="D679" t="inlineStr">
         <is>
-          <t>Fallen Aces</t>
+          <t>Queen's Falls</t>
         </is>
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>Ases Caídos</t>
+          <t>Caídas de la Reina</t>
         </is>
       </c>
       <c r="F679" t="b">

</xml_diff>

<commit_message>
Android: fix Statistics + Localization display bugs (batch 5)
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F703"/>
+  <dimension ref="A1:F704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21639,6 +21639,36 @@
         </is>
       </c>
       <c r="F703" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>beecell_statistics_title</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Stats screen title for Beecell</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Beecell Statistics</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Estadísticas de Beecell</t>
+        </is>
+      </c>
+      <c r="F704" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Localize Casino UI strings
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Localization.xlsx
+++ b/tools/Honeycomb_Localization.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F704"/>
+  <dimension ref="A1:F707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21669,6 +21669,96 @@
         </is>
       </c>
       <c r="F704" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Casino</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>btn_new_bet</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Blackjack action button</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>New Bet</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Nueva Apuesta</t>
+        </is>
+      </c>
+      <c r="F705" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Casino</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>btn_rebuy</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Casino action button to rebuy chips</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Rebuy</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Recomprar</t>
+        </is>
+      </c>
+      <c r="F706" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Casino</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>btn_re_deal</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Blackjack action button to deal again</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Re-Deal</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Repartir</t>
+        </is>
+      </c>
+      <c r="F707" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>